<commit_message>
Uppdateringar utifrån återkoppling från Gunilla och Anna.
</commit_message>
<xml_diff>
--- a/app/data/sni_branschgrupp.xlsx
+++ b/app/data/sni_branschgrupp.xlsx
@@ -533,13 +533,11 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Branschgrupp</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Antal koder</t>
-        </is>
+          <t>Övrigt</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>597</v>
       </c>
     </row>
     <row r="7">
@@ -555,11 +553,11 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Övrigt</t>
+          <t>Livsmedel &amp; dryck</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>598</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8">
@@ -575,11 +573,11 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Livsmedel &amp; dryck</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9">
@@ -620,11 +618,11 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Kemi &amp; material</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12">
@@ -640,11 +638,11 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Kemi &amp; material</t>
+          <t>Papper &amp; förpackning</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13">
@@ -660,11 +658,11 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Metall &amp; stål</t>
+          <t>Trä &amp; trävaror</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -680,11 +678,11 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Papper &amp; förpackning</t>
+          <t>Elkomponenter &amp; energisystem</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -700,11 +698,11 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Trä &amp; trävaror</t>
+          <t>Övrig tillverkning &amp; design</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -720,11 +718,11 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Elkomponenter &amp; energisystem</t>
+          <t>Elektronik &amp; styrsystem</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
@@ -735,36 +733,28 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Huvudgrupp 24</t>
+          <t>Huvudgrupp 24 + 25 (klustrad med Metallprodukter &amp; komponenter, 2026-07-02)</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Övrig tillverkning &amp; design</t>
+          <t>IT &amp; digitala tjänster</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Metallprodukter &amp; komponenter</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Huvudgrupp 25</t>
-        </is>
-      </c>
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="5" t="n"/>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Elektronik &amp; styrsystem</t>
+          <t>Grafiskt &amp; förpackningstryck</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
@@ -780,11 +770,11 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>IT &amp; digitala tjänster</t>
+          <t>Plast &amp; gummi</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
@@ -800,7 +790,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Grafiskt &amp; förpackningstryck</t>
+          <t>Fordonsindustri &amp; bildelar</t>
         </is>
       </c>
       <c r="E20" s="5" t="n">
@@ -820,7 +810,7 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Plast &amp; gummi</t>
+          <t>Möbler &amp; inredning</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
@@ -840,11 +830,11 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Fordonsindustri &amp; bildelar</t>
+          <t>Medtech &amp; vårdteknik</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -860,11 +850,11 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Möbler &amp; inredning</t>
+          <t>Outdoor, sport &amp; fritid</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -880,11 +870,11 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Medtech &amp; vårdteknik</t>
+          <t>Byggsystem &amp; prefabricerat</t>
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -898,14 +888,8 @@
           <t>Huvudgrupp 13, 14, 15</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>Outdoor, sport &amp; fritid</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>2</v>
-      </c>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -918,14 +902,8 @@
           <t>Huvudgrupp 62, 63</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>Byggsystem &amp; prefabricerat</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -947,7 +925,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>32.30 (sportartiklar) + 30.92 (cyklar)</t>
+          <t>32.30 (sportartiklar) + 30.92 (cyklar) + 46.491 (partihandel sport-/fritidsartiklar, klustrad 2026-07-02)</t>
         </is>
       </c>
     </row>
@@ -5215,7 +5193,7 @@
       </c>
       <c r="C230" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D230" s="6" t="n"/>
@@ -5233,7 +5211,7 @@
       </c>
       <c r="C231" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D231" s="6" t="n"/>
@@ -5251,7 +5229,7 @@
       </c>
       <c r="C232" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D232" s="6" t="n"/>
@@ -5269,7 +5247,7 @@
       </c>
       <c r="C233" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D233" s="6" t="n"/>
@@ -5287,7 +5265,7 @@
       </c>
       <c r="C234" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D234" s="6" t="n"/>
@@ -5305,7 +5283,7 @@
       </c>
       <c r="C235" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D235" s="6" t="n"/>
@@ -5323,7 +5301,7 @@
       </c>
       <c r="C236" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D236" s="6" t="n"/>
@@ -5341,7 +5319,7 @@
       </c>
       <c r="C237" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D237" s="6" t="n"/>
@@ -5359,7 +5337,7 @@
       </c>
       <c r="C238" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D238" s="6" t="n"/>
@@ -5377,7 +5355,7 @@
       </c>
       <c r="C239" s="12" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D239" s="12" t="inlineStr">
@@ -5399,7 +5377,7 @@
       </c>
       <c r="C240" s="12" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D240" s="12" t="inlineStr">
@@ -5421,7 +5399,7 @@
       </c>
       <c r="C241" s="12" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D241" s="12" t="inlineStr">
@@ -5443,7 +5421,7 @@
       </c>
       <c r="C242" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D242" s="6" t="n"/>
@@ -5461,7 +5439,7 @@
       </c>
       <c r="C243" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D243" s="6" t="n"/>
@@ -5479,7 +5457,7 @@
       </c>
       <c r="C244" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D244" s="6" t="n"/>
@@ -5497,7 +5475,7 @@
       </c>
       <c r="C245" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D245" s="6" t="n"/>
@@ -5515,7 +5493,7 @@
       </c>
       <c r="C246" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D246" s="6" t="n"/>
@@ -5533,7 +5511,7 @@
       </c>
       <c r="C247" s="6" t="inlineStr">
         <is>
-          <t>Metallprodukter &amp; komponenter</t>
+          <t>Metall &amp; stål</t>
         </is>
       </c>
       <c r="D247" s="6" t="n"/>
@@ -8671,10 +8649,14 @@
       </c>
       <c r="C420" s="9" t="inlineStr">
         <is>
-          <t>Övrigt</t>
-        </is>
-      </c>
-      <c r="D420" s="9" t="n"/>
+          <t>Outdoor, sport &amp; fritid</t>
+        </is>
+      </c>
+      <c r="D420" s="9" t="inlineStr">
+        <is>
+          <t>Klustrad med Outdoor/sportartiklar-tillverkning (2026-07-02).</t>
+        </is>
+      </c>
     </row>
     <row r="421">
       <c r="A421" s="8" t="inlineStr">

</xml_diff>